<commit_message>
Disable old news posts
</commit_message>
<xml_diff>
--- a/out/data/info.xlsx
+++ b/out/data/info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pires\ciampitti-lab.github.io\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{714C491D-1552-4706-AF24-4EC75CCAA910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13BEAF40-796D-4B37-A40C-2DD1707B24FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{680A29BD-E113-4DFE-A325-D924D35BBF8F}"/>
   </bookViews>
@@ -395,9 +395,6 @@
     <t>Prashant’s doctoral research focuses on soil dynamic properties under varying management intensities across North Dakota. His study emphasizes the long-term benefits of minimal soil disturbance and the response of different soil series to these management practices.</t>
   </si>
   <si>
-    <t>Ellayna's research examines the effects of land use—such as conventional tillage in agriculture (full till), conservation practices (minimal till or multi-cropping), and undisturbed systems (native prairies and grasslands)—on soil and water dynamics. Through this work, she aims to identify reliable indicators to define and predict soil health.</t>
-  </si>
-  <si>
     <t>Luis is an intern student at the Pires Lab, taking part in several research projects, such as cover crop seeding and timing methods.</t>
   </si>
   <si>
@@ -410,9 +407,6 @@
     <t>Dr. Pires' research focuses on regenerative agriculture, soil health and nutrient management for building resilient and sustainable agroecossystems.</t>
   </si>
   <si>
-    <t xml:space="preserve">Karen's research focusing on soil health under different soil management systems. Her research explores the long-term impacts of tillage practices, crop rotations and nitrogen sources on soil chemical, physical and biological indicator after 37 years of continuous soil building. </t>
-  </si>
-  <si>
     <t>https://www.linkedin.com/in/luisfbpires/</t>
   </si>
   <si>
@@ -447,6 +441,12 @@
   </si>
   <si>
     <t>group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Karen's research explores the long-term impacts of tillage practices, crop rotations and nitrogen sources on soil chemical, physical and biological indicator after 37 years of continuous soil building. </t>
+  </si>
+  <si>
+    <t>Ellayna's research examines the effects of land use on soil and water dynamics. Through this work, she aims to identify reliable indicators to define and predict soil health.</t>
   </si>
 </sst>
 </file>
@@ -860,7 +860,7 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -874,16 +874,16 @@
         <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>110</v>
       </c>
       <c r="F2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -903,10 +903,10 @@
         <v>111</v>
       </c>
       <c r="F3" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="G3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -929,7 +929,7 @@
         <v>118</v>
       </c>
       <c r="G4" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -949,10 +949,10 @@
         <v>113</v>
       </c>
       <c r="F5" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="G5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -966,7 +966,7 @@
         <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E6" t="s">
         <v>114</v>
@@ -975,7 +975,7 @@
         <v>117</v>
       </c>
       <c r="G6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -995,10 +995,10 @@
         <v>115</v>
       </c>
       <c r="F7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1015,13 +1015,13 @@
         <v>108</v>
       </c>
       <c r="E8" t="s">
+        <v>123</v>
+      </c>
+      <c r="F8" t="s">
+        <v>119</v>
+      </c>
+      <c r="G8" t="s">
         <v>125</v>
-      </c>
-      <c r="F8" t="s">
-        <v>120</v>
-      </c>
-      <c r="G8" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1041,10 +1041,10 @@
         <v>116</v>
       </c>
       <c r="F9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1052,16 +1052,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C10" t="s">
         <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="G10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1069,16 +1069,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C11" t="s">
         <v>3</v>
       </c>
       <c r="D11" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G11" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1086,17 +1086,17 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C12" t="s">
         <v>3</v>
       </c>
       <c r="D12" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E12" s="1"/>
       <c r="G12" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
renewing and updating the hole website
</commit_message>
<xml_diff>
--- a/out/data/info.xlsx
+++ b/out/data/info.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pires\ciampitti-lab.github.io\public\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pires\pires-lab.github.io\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13BEAF40-796D-4B37-A40C-2DD1707B24FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D73F82B-ECF0-4572-A858-565F8D75A256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{680A29BD-E113-4DFE-A325-D924D35BBF8F}"/>
   </bookViews>
@@ -395,15 +395,6 @@
     <t>Prashant’s doctoral research focuses on soil dynamic properties under varying management intensities across North Dakota. His study emphasizes the long-term benefits of minimal soil disturbance and the response of different soil series to these management practices.</t>
   </si>
   <si>
-    <t>Luis is an intern student at the Pires Lab, taking part in several research projects, such as cover crop seeding and timing methods.</t>
-  </si>
-  <si>
-    <t>Maria Eduarda is now an student intern at the Pires Lab, contributing to several research projects.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marcos supports multiple research and extension projects throughout North Dakota as a student intern. </t>
-  </si>
-  <si>
     <t>Dr. Pires' research focuses on regenerative agriculture, soil health and nutrient management for building resilient and sustainable agroecossystems.</t>
   </si>
   <si>
@@ -443,17 +434,26 @@
     <t>group</t>
   </si>
   <si>
-    <t xml:space="preserve">Karen's research explores the long-term impacts of tillage practices, crop rotations and nitrogen sources on soil chemical, physical and biological indicator after 37 years of continuous soil building. </t>
-  </si>
-  <si>
     <t>Ellayna's research examines the effects of land use on soil and water dynamics. Through this work, she aims to identify reliable indicators to define and predict soil health.</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/thassiany-de-castro-alves-13a148346/</t>
+  </si>
+  <si>
+    <t>https://br.linkedin.com/in/marcos-centuri%C3%B3n-900202281</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/artur-carmona-800214403</t>
+  </si>
+  <si>
+    <t>Artur Carmona is an Agronomy student at the Federal University of Rio Grande do Sul (UFRGS). To complement his academic training and gain a broader understanding of global agriculture, he is currently conducting an internship at North Dakota State University (NDSU).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -468,6 +468,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -491,9 +497,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -860,7 +867,7 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -874,16 +881,16 @@
         <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>110</v>
       </c>
       <c r="F2" t="s">
+        <v>119</v>
+      </c>
+      <c r="G2" t="s">
         <v>122</v>
-      </c>
-      <c r="G2" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -902,11 +909,8 @@
       <c r="E3" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="F3" t="s">
-        <v>135</v>
-      </c>
       <c r="G3" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -929,7 +933,7 @@
         <v>118</v>
       </c>
       <c r="G4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -949,10 +953,10 @@
         <v>113</v>
       </c>
       <c r="F5" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="G5" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -966,7 +970,7 @@
         <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E6" t="s">
         <v>114</v>
@@ -975,7 +979,7 @@
         <v>117</v>
       </c>
       <c r="G6" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -994,11 +998,8 @@
       <c r="E7" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="F7" t="s">
-        <v>121</v>
-      </c>
       <c r="G7" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1015,13 +1016,10 @@
         <v>108</v>
       </c>
       <c r="E8" t="s">
-        <v>123</v>
-      </c>
-      <c r="F8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G8" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1040,28 +1038,29 @@
       <c r="E9" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F9" t="s">
-        <v>120</v>
-      </c>
       <c r="G9" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C10" t="s">
         <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>130</v>
-      </c>
+        <v>127</v>
+      </c>
+      <c r="E10" t="s">
+        <v>133</v>
+      </c>
+      <c r="F10" s="2"/>
       <c r="G10" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1069,16 +1068,22 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C11" t="s">
         <v>3</v>
       </c>
       <c r="D11" t="s">
-        <v>133</v>
+        <v>130</v>
+      </c>
+      <c r="E11" t="s">
+        <v>135</v>
+      </c>
+      <c r="F11" t="s">
+        <v>136</v>
       </c>
       <c r="G11" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1086,17 +1091,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C12" t="s">
         <v>3</v>
       </c>
       <c r="D12" t="s">
-        <v>129</v>
-      </c>
-      <c r="E12" s="1"/>
+        <v>126</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>134</v>
+      </c>
       <c r="G12" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>